<commit_message>
garth script fr folder to snowflake
</commit_message>
<xml_diff>
--- a/load_errors/EOM_Transactions_202501_errors.xlsx
+++ b/load_errors/EOM_Transactions_202501_errors.xlsx
@@ -425,34 +425,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:A2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Source File</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Excel Row Number</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Error Description</t>
+          <t>ERROR_DESCRIPTION</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
-        <is>
-          <t>C:\ETL\EOM PYTHON SCRIPTS\2025 EOM Reports-20260923T222736Z-1-002\2025 EOM Reports\2025-01 EOM Reports\EOM Transactions - 202501.xlsx</t>
-        </is>
-      </c>
-      <c r="B2" t="inlineStr"/>
-      <c r="C2" t="inlineStr">
         <is>
           <t>Duplicate column name(s): Total Treaty</t>
         </is>

</xml_diff>